<commit_message>
demo update, script/package/dependencies updater added
</commit_message>
<xml_diff>
--- a/demo 2 (alpha)/Pb210_results/CA modeling data/elogpb210_md_CA_summary.xlsx
+++ b/demo 2 (alpha)/Pb210_results/CA modeling data/elogpb210_md_CA_summary.xlsx
@@ -403,19 +403,19 @@
         </is>
       </c>
       <c r="C2">
-        <v>2.685104549724821</v>
+        <v>2.687373770362765</v>
       </c>
       <c r="D2">
-        <v>0.06382876700337205</v>
+        <v>0.06476012359947618</v>
       </c>
       <c r="E2">
-        <v>42.06731033333243</v>
+        <v>41.49735394242672</v>
       </c>
       <c r="F2">
-        <v>2.992828943636855E-30</v>
+        <v>4.65651889170438E-30</v>
       </c>
       <c r="G2">
-        <v>0.9495650606717169</v>
+        <v>0.9486982531502455</v>
       </c>
     </row>
     <row r="3">
@@ -430,19 +430,19 @@
         </is>
       </c>
       <c r="C3">
-        <v>-0.2812607486159102</v>
+        <v>-0.2828185164766085</v>
       </c>
       <c r="D3">
-        <v>0.01110795475610751</v>
+        <v>0.0112700363286809</v>
       </c>
       <c r="E3">
-        <v>-25.32066026477682</v>
+        <v>-25.09472979753127</v>
       </c>
       <c r="F3">
-        <v>3.394715191626438E-23</v>
+        <v>4.498780282866806E-23</v>
       </c>
       <c r="G3">
-        <v>0.9495650606717169</v>
+        <v>0.9486982531502455</v>
       </c>
     </row>
   </sheetData>

</xml_diff>